<commit_message>
the finished workbooks with his critique applied: every column a measure he named (times, tokens, runtime, build cost, the RAGAS scores) or an id; the interpreter named as he names it; tries, cached tokens, request counts, load times and the three kinds of build seconds taken out; the judge's cost in the run sheet as the evaluation's own
</commit_message>
<xml_diff>
--- a/finished_data/artefact_construction.xlsx
+++ b/finished_data/artefact_construction.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'build'!$A$1:$N$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'index'!$A$1:$B$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'key'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'build'!$A$1:$I$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'index'!$A$1:$B$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'key'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -432,14 +432,9 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="27" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,47 +465,22 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>calls</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>count_of</t>
+          <t>tokens_in</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>calls</t>
+          <t>tokens_out</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>tries</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>tokens_in</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>tokens_out</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>seconds_start_to_end</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>seconds_of_calls_added_up</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>seconds_of_the_whole_command</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
@@ -535,14 +505,6 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>5843</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>chunks</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -565,14 +527,6 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>974</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>chunks</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -601,30 +555,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>5843</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>chunks</t>
-        </is>
+        <v>5826</v>
+      </c>
+      <c r="G4" t="n">
+        <v>9854855</v>
       </c>
       <c r="H4" t="n">
-        <v>5826</v>
+        <v>1841463</v>
       </c>
       <c r="I4" t="n">
-        <v>5891</v>
-      </c>
-      <c r="J4" t="n">
-        <v>9854855</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1841463</v>
-      </c>
-      <c r="L4" t="n">
         <v>4224.8</v>
-      </c>
-      <c r="M4" t="n">
-        <v>16896.2</v>
       </c>
     </row>
     <row r="5">
@@ -656,28 +596,14 @@
       <c r="F5" t="n">
         <v>5817</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>chunks</t>
-        </is>
+      <c r="G5" t="n">
+        <v>11889245</v>
       </c>
       <c r="H5" t="n">
-        <v>5817</v>
+        <v>8033494</v>
       </c>
       <c r="I5" t="n">
-        <v>5817</v>
-      </c>
-      <c r="J5" t="n">
-        <v>11889245</v>
-      </c>
-      <c r="K5" t="n">
-        <v>8033494</v>
-      </c>
-      <c r="L5" t="n">
         <v>9183.6</v>
-      </c>
-      <c r="M5" t="n">
-        <v>36718.1</v>
       </c>
     </row>
     <row r="6">
@@ -709,28 +635,14 @@
       <c r="F6" t="n">
         <v>33</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>files</t>
-        </is>
+      <c r="G6" t="n">
+        <v>492482</v>
       </c>
       <c r="H6" t="n">
-        <v>33</v>
+        <v>6252</v>
       </c>
       <c r="I6" t="n">
-        <v>33</v>
-      </c>
-      <c r="J6" t="n">
-        <v>492482</v>
-      </c>
-      <c r="K6" t="n">
-        <v>6252</v>
-      </c>
-      <c r="L6" t="n">
         <v>25.5</v>
-      </c>
-      <c r="M6" t="n">
-        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -762,28 +674,14 @@
       <c r="F7" t="n">
         <v>33</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>files</t>
-        </is>
+      <c r="G7" t="n">
+        <v>500153</v>
       </c>
       <c r="H7" t="n">
-        <v>33</v>
+        <v>114902</v>
       </c>
       <c r="I7" t="n">
-        <v>33</v>
-      </c>
-      <c r="J7" t="n">
-        <v>500153</v>
-      </c>
-      <c r="K7" t="n">
-        <v>114902</v>
-      </c>
-      <c r="L7" t="n">
         <v>123.3</v>
-      </c>
-      <c r="M7" t="n">
-        <v>466.6</v>
       </c>
     </row>
     <row r="8">
@@ -812,20 +710,17 @@
           <t>Anthropic API, 4 calls at a time</t>
         </is>
       </c>
+      <c r="F8" t="n">
+        <v>26</v>
+      </c>
+      <c r="G8" t="n">
+        <v>44008</v>
+      </c>
       <c r="H8" t="n">
-        <v>26</v>
-      </c>
-      <c r="J8" t="n">
-        <v>44008</v>
-      </c>
-      <c r="K8" t="n">
         <v>9158</v>
       </c>
-      <c r="L8" t="n">
+      <c r="I8" t="n">
         <v>19.9</v>
-      </c>
-      <c r="M8" t="n">
-        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -854,20 +749,17 @@
           <t>Anthropic API, 4 calls at a time</t>
         </is>
       </c>
+      <c r="F9" t="n">
+        <v>26</v>
+      </c>
+      <c r="G9" t="n">
+        <v>53241</v>
+      </c>
       <c r="H9" t="n">
-        <v>26</v>
-      </c>
-      <c r="J9" t="n">
-        <v>53241</v>
-      </c>
-      <c r="K9" t="n">
         <v>37542</v>
       </c>
-      <c r="L9" t="n">
+      <c r="I9" t="n">
         <v>45.3</v>
-      </c>
-      <c r="M9" t="n">
-        <v>167.7</v>
       </c>
     </row>
     <row r="10">
@@ -896,20 +788,17 @@
           <t>Anthropic API, 4 calls at a time</t>
         </is>
       </c>
+      <c r="F10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>130756</v>
+      </c>
       <c r="H10" t="n">
-        <v>7</v>
-      </c>
-      <c r="J10" t="n">
-        <v>130756</v>
-      </c>
-      <c r="K10" t="n">
         <v>31445</v>
       </c>
-      <c r="L10" t="n">
+      <c r="I10" t="n">
         <v>35.7</v>
-      </c>
-      <c r="M10" t="n">
-        <v>120.7</v>
       </c>
     </row>
     <row r="11">
@@ -938,20 +827,17 @@
           <t>Anthropic API, 4 calls at a time</t>
         </is>
       </c>
+      <c r="F11" t="n">
+        <v>17</v>
+      </c>
+      <c r="G11" t="n">
+        <v>17915</v>
+      </c>
       <c r="H11" t="n">
-        <v>17</v>
-      </c>
-      <c r="J11" t="n">
-        <v>17915</v>
-      </c>
-      <c r="K11" t="n">
         <v>884</v>
       </c>
-      <c r="L11" t="n">
+      <c r="I11" t="n">
         <v>4.6</v>
-      </c>
-      <c r="M11" t="n">
-        <v>15.8</v>
       </c>
     </row>
     <row r="12">
@@ -975,7 +861,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="L12" t="n">
+      <c r="I12" t="n">
         <v>1018.9</v>
       </c>
     </row>
@@ -987,7 +873,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tags taken out, with their 5,470 edges</t>
+          <t>4,111 tags taken out, with their 5,470 edges</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1000,15 +886,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>4111</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
+      <c r="I13" t="n">
         <v>9.1</v>
       </c>
     </row>
@@ -1033,7 +911,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="L14" t="n">
+      <c r="I14" t="n">
         <v>193</v>
       </c>
     </row>
@@ -1058,7 +936,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="I15" t="n">
         <v>6.8</v>
       </c>
     </row>
@@ -1083,7 +961,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="L16" t="n">
+      <c r="I16" t="n">
         <v>42.3</v>
       </c>
     </row>
@@ -1116,24 +994,13 @@
       <c r="F17" t="n">
         <v>16714</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>texts</t>
-        </is>
+      <c r="G17" t="n">
+        <v>103614</v>
       </c>
       <c r="H17" t="n">
-        <v>16714</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>16714</v>
-      </c>
-      <c r="J17" t="n">
-        <v>103614</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
         <v>511.5</v>
       </c>
     </row>
@@ -1166,24 +1033,13 @@
       <c r="F18" t="n">
         <v>63</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>texts</t>
-        </is>
+      <c r="G18" t="n">
+        <v>583</v>
       </c>
       <c r="H18" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>63</v>
-      </c>
-      <c r="J18" t="n">
-        <v>583</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
         <v>19.2</v>
       </c>
     </row>
@@ -1216,24 +1072,13 @@
       <c r="F19" t="n">
         <v>4869</v>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>texts</t>
-        </is>
+      <c r="G19" t="n">
+        <v>351855</v>
       </c>
       <c r="H19" t="n">
-        <v>4869</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>4869</v>
-      </c>
-      <c r="J19" t="n">
-        <v>351855</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
         <v>287.5</v>
       </c>
     </row>
@@ -1258,15 +1103,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>16714</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>vectors</t>
-        </is>
-      </c>
-      <c r="L20" t="n">
+      <c r="I20" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1291,15 +1128,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>4869</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>vectors</t>
-        </is>
-      </c>
-      <c r="L21" t="n">
+      <c r="I21" t="n">
         <v>73</v>
       </c>
     </row>
@@ -1332,25 +1161,14 @@
       <c r="F22" t="n">
         <v>420</v>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>pairs</t>
-        </is>
+      <c r="G22" t="n">
+        <v>14256990</v>
       </c>
       <c r="H22" t="n">
-        <v>420</v>
-      </c>
-      <c r="J22" t="n">
-        <v>14256990</v>
-      </c>
-      <c r="K22" t="n">
         <v>15982</v>
       </c>
-      <c r="L22" t="n">
+      <c r="I22" t="n">
         <v>642.9</v>
-      </c>
-      <c r="M22" t="n">
-        <v>5101.1</v>
       </c>
     </row>
     <row r="23">
@@ -1382,25 +1200,14 @@
       <c r="F23" t="n">
         <v>500</v>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>pairs</t>
-        </is>
+      <c r="G23" t="n">
+        <v>16981038</v>
       </c>
       <c r="H23" t="n">
-        <v>500</v>
-      </c>
-      <c r="J23" t="n">
-        <v>16981038</v>
-      </c>
-      <c r="K23" t="n">
         <v>19089</v>
       </c>
-      <c r="L23" t="n">
+      <c r="I23" t="n">
         <v>815.7</v>
-      </c>
-      <c r="M23" t="n">
-        <v>6479.9</v>
       </c>
     </row>
     <row r="24">
@@ -1432,22 +1239,11 @@
       <c r="F24" t="n">
         <v>72</v>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>pairs</t>
-        </is>
+      <c r="G24" t="n">
+        <v>2441986</v>
       </c>
       <c r="H24" t="n">
-        <v>72</v>
-      </c>
-      <c r="J24" t="n">
-        <v>2441986</v>
-      </c>
-      <c r="K24" t="n">
         <v>2718</v>
-      </c>
-      <c r="M24" t="n">
-        <v>1185.4</v>
       </c>
     </row>
     <row r="25">
@@ -1479,25 +1275,14 @@
       <c r="F25" t="n">
         <v>728</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>pairs</t>
-        </is>
+      <c r="G25" t="n">
+        <v>24725666</v>
       </c>
       <c r="H25" t="n">
-        <v>728</v>
-      </c>
-      <c r="J25" t="n">
-        <v>24725666</v>
-      </c>
-      <c r="K25" t="n">
         <v>27807</v>
       </c>
-      <c r="L25" t="n">
+      <c r="I25" t="n">
         <v>1105.8</v>
-      </c>
-      <c r="M25" t="n">
-        <v>8786.200000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1508,7 +1293,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>encoder candidate: the bake-off's edges encoded</t>
+          <t>encoder candidate: 5,469 edges encoded for the bake-off</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1526,18 +1311,10 @@
           <t>Colab, NVIDIA GPU (CUDA)</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>5469</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="K26" t="n">
+      <c r="H26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="n">
+      <c r="I26" t="n">
         <v>430.3</v>
       </c>
     </row>
@@ -1549,7 +1326,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>encoder candidate: the bake-off's edges encoded</t>
+          <t>encoder candidate: 5,469 edges encoded for the bake-off</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1567,18 +1344,10 @@
           <t>Colab, NVIDIA GPU (CUDA)</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>5469</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
+      <c r="H27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="n">
+      <c r="I27" t="n">
         <v>792.8</v>
       </c>
     </row>
@@ -1590,7 +1359,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>encoder candidate: the bake-off's edges encoded</t>
+          <t>encoder candidate: 5,469 edges encoded for the bake-off</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1608,18 +1377,10 @@
           <t>Colab, NVIDIA GPU (CUDA)</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>5469</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="K28" t="n">
+      <c r="H28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="n">
+      <c r="I28" t="n">
         <v>728.4</v>
       </c>
     </row>
@@ -1631,7 +1392,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>encoder candidate: the bake-off's edges encoded</t>
+          <t>encoder candidate: 5,469 edges encoded for the bake-off</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1649,18 +1410,10 @@
           <t>Colab, NVIDIA GPU (CUDA)</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>5469</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="K29" t="n">
+      <c r="H29" t="n">
         <v>0</v>
       </c>
-      <c r="L29" t="n">
+      <c r="I29" t="n">
         <v>1275.5</v>
       </c>
     </row>
@@ -1685,7 +1438,7 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="L30" t="n">
+      <c r="I30" t="n">
         <v>2069.2</v>
       </c>
     </row>
@@ -1715,18 +1468,10 @@
           <t>desktop, NVIDIA GeForce GTX 1080 Ti</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>61018</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="K31" t="n">
+      <c r="H31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="n">
+      <c r="I31" t="n">
         <v>3549.5</v>
       </c>
     </row>
@@ -1751,15 +1496,7 @@
           <t>laptop CPU</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>27</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>combinations fitted</t>
-        </is>
-      </c>
-      <c r="L32" t="n">
+      <c r="I32" t="n">
         <v>979.4</v>
       </c>
     </row>
@@ -1771,7 +1508,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>bootstrap refits of the head</t>
+          <t>24 bootstrap refits of the head</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1784,15 +1521,7 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>24</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>refits</t>
-        </is>
-      </c>
-      <c r="L33" t="n">
+      <c r="I33" t="n">
         <v>99</v>
       </c>
     </row>
@@ -1817,7 +1546,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="L34" t="n">
+      <c r="I34" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1842,15 +1571,7 @@
           <t>Neo4j on the laptop</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>61018</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="L35" t="n">
+      <c r="I35" t="n">
         <v>91</v>
       </c>
     </row>
@@ -1875,15 +1596,7 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>26950</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>edges</t>
-        </is>
-      </c>
-      <c r="N36" t="n">
+      <c r="I36" t="n">
         <v>35.2</v>
       </c>
     </row>
@@ -1908,15 +1621,7 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>1043</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>customer-to-chunk edges</t>
-        </is>
-      </c>
-      <c r="N37" t="n">
+      <c r="I37" t="n">
         <v>67</v>
       </c>
     </row>
@@ -1941,20 +1646,12 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>38377</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>times</t>
-        </is>
-      </c>
-      <c r="N38" t="n">
+      <c r="I38" t="n">
         <v>9.5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N38"/>
+  <autoFilter ref="A1:I38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1965,7 +1662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1987,77 +1684,77 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Channel nodes</t>
+          <t>files</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>302</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chunk nodes</t>
+          <t>products</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4869</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Company nodes</t>
+          <t>channels</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Customer nodes</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120</v>
+        <v>530</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Employee nodes</t>
+          <t>customers</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>530</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FacetLayer nodes</t>
+          <t>companies</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>File nodes</t>
+          <t>record kinds</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kind nodes</t>
+          <t>organisations</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2067,37 +1764,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Org nodes</t>
+          <t>roles</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Product nodes</t>
+          <t>chunks in the graph</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>4869</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Role nodes</t>
+          <t>chunks the arm searches</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>17</v>
+        <v>4808</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tag nodes</t>
+          <t>tags in the graph</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2107,17 +1804,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>(File)-[HAS_CHUNK]-&gt;(Chunk) relationships</t>
+          <t>tags on the chunks the arm searches</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4869</v>
+        <v>16654</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(Chunk)-[HAS_TAG]-&gt;(Tag) relationships</t>
+          <t>tag-to-chunk edges in the graph</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2127,27 +1824,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(Chunk)-[channel]-&gt;(Channel) relationships</t>
+          <t>tag-to-chunk edges on the chunks the arm searches</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2677</v>
+        <v>61018</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(File)-[channel]-&gt;(Channel) relationships</t>
+          <t>person-to-chunk edges</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>302</v>
+        <v>26950</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(Customer)-[chunk]-&gt;(Chunk) relationships</t>
+          <t>customer-to-chunk edges</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2157,345 +1854,15 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(Employee)-[chunk]-&gt;(Chunk) relationships</t>
+          <t>chunks with their records' times</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>26950</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>(Customer)-[company]-&gt;(Company) relationships</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>(File)-[company]-&gt;(Company) relationships</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>(File)-[customer]-&gt;(Customer) relationships</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>(Employee)-[documents]-&gt;(Product) relationships</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>(File)-[employee]-&gt;(Employee) relationships</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1060</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>(Product)-[has]-&gt;(Kind) relationships</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>(Chunk)-[kind]-&gt;(Kind) relationships</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>4808</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>(Employee)-[manages]-&gt;(Employee) relationships</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>(Employee)-[meeting_transcripts]-&gt;(Product) relationships</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>(Employee)-[org]-&gt;(Org) relationships</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>(File)-[org]-&gt;(Org) relationships</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>(Chunk)-[product]-&gt;(Product) relationships</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>4808</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>(File)-[product]-&gt;(Product) relationships</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>(Customer)-[role]-&gt;(Role) relationships</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>(Employee)-[role]-&gt;(Role) relationships</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>(File)-[role]-&gt;(Role) relationships</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>(Employee)-[slack]-&gt;(Channel) relationships</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>2647</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>(Product)-[slack]-&gt;(Channel) relationships</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>chunks the arm reads</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>4808</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>tags on those chunks</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>16654</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>tag-to-chunk edges on those chunks</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>61018</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>tags compared with the question's tags</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>16609</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>edges of those tags</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>57204</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>products</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>people of the products</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>1307</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>channels apart from their product</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>chunks with their records' times</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
         <v>4747</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Channel nodes with a name</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Company nodes with a name</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Customer nodes with a name</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Employee nodes with a name</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Product nodes with a name</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>tokens of all chunks, the chunker's estimate</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>3850319</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B52"/>
+  <autoFilter ref="A1:B19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2506,11 +1873,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="100" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -2639,12 +2006,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>calls</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>How many things the part made or handled. Empty where not counted.</t>
+          <t>Calls to a language model that gave an answer, or requests to an embedding model. Empty where the part made no calls, or where they were not counted.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2661,15 +2028,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>count_of</t>
+          <t>tokens_in</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>What count counts.</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>Tokens sent to the model. Empty where not counted.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>tokens</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2679,17 +2050,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>calls</t>
+          <t>tokens_out</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Calls to a language model that gave an answer, or requests to an embedding model.</t>
+          <t>Tokens that the model wrote. 0 for an embedding model or an encoder.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>tokens</t>
         </is>
       </c>
     </row>
@@ -2701,172 +2072,62 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tries</t>
+          <t>seconds</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Every try of those calls, failed tries included. Empty where the tries were not counted.</t>
+          <t>Time of the part, from its start to its end. Empty where not measured.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>seconds</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>index</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tokens_in</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tokens sent to the model.</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>tokens</t>
-        </is>
-      </c>
+          <t>What the index holds.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>index</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>tokens_out</t>
+          <t>value</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tokens that the model wrote. 0 for an embedding model or an encoder.</t>
+          <t>How many.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>build</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>seconds_start_to_end</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Time from the start to the end of the part. Empty where not measured.</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>build</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>seconds_of_calls_added_up</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>The time of each call, added up. With several calls at the same time, it is more than seconds_start_to_end. Empty where not measured.</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>build</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>seconds_of_the_whole_command</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Time of the whole command that made the part, its backup and check included. Empty where not measured.</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>seconds</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>What is counted.</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>The count.</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
           <t>count</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D17"/>
+  <autoFilter ref="A1:D12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>